<commit_message>
feat(sheets): 민요 신규 곡 봄철나비 (4/4 16정간)
</commit_message>
<xml_diff>
--- a/sheets/민요/검수/_목록.xlsx
+++ b/sheets/민요/검수/_목록.xlsx
@@ -5056,8 +5056,53 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" s="2">
+        <v>87</v>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">봄철나비.csv</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">봄철나비</t>
+        </is>
+      </c>
+      <c r="D88" s="4"/>
+      <c r="E88" s="2"/>
+      <c r="F88" s="2"/>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4/4</t>
+        </is>
+      </c>
+      <c r="H88" s="2">
+        <v>16</v>
+      </c>
+      <c r="I88" s="2">
+        <v>1</v>
+      </c>
+      <c r="J88" s="2">
+        <v>47</v>
+      </c>
+      <c r="K88" s="2">
+        <v>0</v>
+      </c>
+      <c r="L88" s="2">
+        <v>0</v>
+      </c>
+      <c r="M88" s="2"/>
+      <c r="N88" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">검수 xlsx 직접 입력 (거스러미 돈돈날이.xlsx 복사)</t>
+        </is>
+      </c>
+      <c r="O88" s="4"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O87"/>
+  <autoFilter ref="A1:O88"/>
 </worksheet>
 </file>
 

</xml_diff>